<commit_message>
Issue with noise being added to output is fixed!
</commit_message>
<xml_diff>
--- a/Results.xlsx
+++ b/Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\myaze\Desktop\College\Grad\Grad Research\Contact_GNN_From_Scratch\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7E7917A1-FF12-47FF-8758-272032F19DD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{193582ED-E9D5-465C-84B0-FD96F2D33281}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{CB31053B-9DB6-40E9-ACAD-70ACA465CC93}"/>
   </bookViews>
@@ -369,7 +369,7 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr lang="en-US"/>
-                  <a:t>Epoch</a:t>
+                  <a:t>Train Samples</a:t>
                 </a:r>
               </a:p>
             </c:rich>
@@ -855,13 +855,27 @@
               <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
               <a:lstStyle/>
               <a:p>
-                <a:pPr>
+                <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="ctr" defTabSz="914400" rtl="0" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+                  <a:lnSpc>
+                    <a:spcPct val="100000"/>
+                  </a:lnSpc>
+                  <a:spcBef>
+                    <a:spcPts val="0"/>
+                  </a:spcBef>
+                  <a:spcAft>
+                    <a:spcPts val="0"/>
+                  </a:spcAft>
+                  <a:buClrTx/>
+                  <a:buSzTx/>
+                  <a:buFontTx/>
+                  <a:buNone/>
+                  <a:tabLst/>
                   <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
-                      <a:schemeClr val="tx1">
+                      <a:sysClr val="windowText" lastClr="000000">
                         <a:lumMod val="65000"/>
                         <a:lumOff val="35000"/>
-                      </a:schemeClr>
+                      </a:sysClr>
                     </a:solidFill>
                     <a:latin typeface="+mn-lt"/>
                     <a:ea typeface="+mn-ea"/>
@@ -869,8 +883,15 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="en-US"/>
-                  <a:t>Epoch</a:t>
+                  <a:rPr lang="en-US" sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:sysClr val="windowText" lastClr="000000">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:sysClr>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>Train Samples</a:t>
                 </a:r>
               </a:p>
             </c:rich>
@@ -887,13 +908,27 @@
             <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
             <a:lstStyle/>
             <a:p>
-              <a:pPr>
+              <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="ctr" defTabSz="914400" rtl="0" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+                <a:lnSpc>
+                  <a:spcPct val="100000"/>
+                </a:lnSpc>
+                <a:spcBef>
+                  <a:spcPts val="0"/>
+                </a:spcBef>
+                <a:spcAft>
+                  <a:spcPts val="0"/>
+                </a:spcAft>
+                <a:buClrTx/>
+                <a:buSzTx/>
+                <a:buFontTx/>
+                <a:buNone/>
+                <a:tabLst/>
                 <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
-                    <a:schemeClr val="tx1">
+                    <a:sysClr val="windowText" lastClr="000000">
                       <a:lumMod val="65000"/>
                       <a:lumOff val="35000"/>
-                    </a:schemeClr>
+                    </a:sysClr>
                   </a:solidFill>
                   <a:latin typeface="+mn-lt"/>
                   <a:ea typeface="+mn-ea"/>
@@ -1356,13 +1391,27 @@
               <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
               <a:lstStyle/>
               <a:p>
-                <a:pPr>
+                <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="ctr" defTabSz="914400" rtl="0" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+                  <a:lnSpc>
+                    <a:spcPct val="100000"/>
+                  </a:lnSpc>
+                  <a:spcBef>
+                    <a:spcPts val="0"/>
+                  </a:spcBef>
+                  <a:spcAft>
+                    <a:spcPts val="0"/>
+                  </a:spcAft>
+                  <a:buClrTx/>
+                  <a:buSzTx/>
+                  <a:buFontTx/>
+                  <a:buNone/>
+                  <a:tabLst/>
                   <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
-                      <a:schemeClr val="tx1">
+                      <a:sysClr val="windowText" lastClr="000000">
                         <a:lumMod val="65000"/>
                         <a:lumOff val="35000"/>
-                      </a:schemeClr>
+                      </a:sysClr>
                     </a:solidFill>
                     <a:latin typeface="+mn-lt"/>
                     <a:ea typeface="+mn-ea"/>
@@ -1370,8 +1419,15 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="en-US"/>
-                  <a:t>Epoch</a:t>
+                  <a:rPr lang="en-US" sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:sysClr val="windowText" lastClr="000000">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:sysClr>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>Train Samples</a:t>
                 </a:r>
               </a:p>
             </c:rich>
@@ -1388,13 +1444,27 @@
             <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
             <a:lstStyle/>
             <a:p>
-              <a:pPr>
+              <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="ctr" defTabSz="914400" rtl="0" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+                <a:lnSpc>
+                  <a:spcPct val="100000"/>
+                </a:lnSpc>
+                <a:spcBef>
+                  <a:spcPts val="0"/>
+                </a:spcBef>
+                <a:spcAft>
+                  <a:spcPts val="0"/>
+                </a:spcAft>
+                <a:buClrTx/>
+                <a:buSzTx/>
+                <a:buFontTx/>
+                <a:buNone/>
+                <a:tabLst/>
                 <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
-                    <a:schemeClr val="tx1">
+                    <a:sysClr val="windowText" lastClr="000000">
                       <a:lumMod val="65000"/>
                       <a:lumOff val="35000"/>
-                    </a:schemeClr>
+                    </a:sysClr>
                   </a:solidFill>
                   <a:latin typeface="+mn-lt"/>
                   <a:ea typeface="+mn-ea"/>

</xml_diff>